<commit_message>
feat: optimize pxkdl and rebuild import feature on pxldl
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/agent/MauUpload_PXK_HKGDL_TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/agent/MauUpload_PXK_HKGDL_TT78.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
@@ -33,7 +33,24 @@
     <author>ASIA</author>
   </authors>
   <commentList>
-    <comment ref="X1" authorId="0">
+    <comment ref="Z1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="13"/>
+            <rFont val="Times New Roman"/>
+            <charset val="134"/>
+          </rPr>
+          <t>Tính chất hàng hóa, dịch vụ
+1: HH/DV
+2: KM
+3: GK
+4: Ghi chú</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -55,48 +72,60 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="57">
-  <si>
-    <t>Số phiếu(*)</t>
-  </si>
-  <si>
-    <t>Ngày xuất(*)</t>
-  </si>
-  <si>
-    <t>Người điều động(*)</t>
-  </si>
-  <si>
-    <t>Về việc(*)</t>
-  </si>
-  <si>
-    <t>Hợp đồng kinh tế số(*)</t>
-  </si>
-  <si>
-    <t>Hợp đồng kinh tế ngày(*)</t>
-  </si>
-  <si>
-    <t>Người vận chuyển(*)</t>
-  </si>
-  <si>
-    <t>Phương tiện vận chuyển(*)</t>
-  </si>
-  <si>
-    <t>Xuất tại kho - Mã kho(*)</t>
-  </si>
-  <si>
-    <t>Nhập tại kho - Mã kho(*)</t>
-  </si>
-  <si>
-    <t>MST người xuất</t>
-  </si>
-  <si>
-    <t>Họ và tên người xuất</t>
-  </si>
-  <si>
-    <t>Tên đơn vị</t>
-  </si>
-  <si>
-    <t>Email nhận</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="63">
+  <si>
+    <t>Mã phiếu(*)</t>
+  </si>
+  <si>
+    <t>Địa chỉ xuất kho (*)</t>
+  </si>
+  <si>
+    <t>Ngày lập (*)</t>
+  </si>
+  <si>
+    <t>Họ và tên người xuất kho (*)</t>
+  </si>
+  <si>
+    <t>Loại tiền (*)</t>
+  </si>
+  <si>
+    <t>Tên người vận chuyển (*)</t>
+  </si>
+  <si>
+    <t>Hợp đồng kinh tế số (*)</t>
+  </si>
+  <si>
+    <t>Hợp đồng kinh tế ngày (*)</t>
+  </si>
+  <si>
+    <t>Phương tiện vận chuyển (*)</t>
+  </si>
+  <si>
+    <t>Mã số thuế người nhập</t>
+  </si>
+  <si>
+    <t>Họ và Tên người nhập</t>
+  </si>
+  <si>
+    <t>Tên đơn vị nhập</t>
+  </si>
+  <si>
+    <t>Địa chỉ nhập kho (*)</t>
+  </si>
+  <si>
+    <t>Nội dung nhập kho</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Số điện thoại</t>
+  </si>
+  <si>
+    <t>Số tài khoản</t>
+  </si>
+  <si>
+    <t>Tại ngân hàng</t>
   </si>
   <si>
     <t>STT(*)</t>
@@ -111,10 +140,7 @@
     <t>Đơn vị tính</t>
   </si>
   <si>
-    <t>Thực xuất(*)</t>
-  </si>
-  <si>
-    <t>Thực nhập</t>
+    <t>Số lượng(*)</t>
   </si>
   <si>
     <t>Đơn giá(*)</t>
@@ -123,40 +149,40 @@
     <t>Thành tiền(*)</t>
   </si>
   <si>
-    <t>Tổng tiền(*)</t>
-  </si>
-  <si>
     <t>Tính Chất(*)</t>
   </si>
   <si>
-    <t>Số tiền bằng chữ</t>
+    <t>Tỷ giá(*)</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>03/03/2023</t>
+    <t>Địa chỉ xuất kho 1</t>
+  </si>
+  <si>
+    <t>12/05/2026</t>
   </si>
   <si>
     <t>Nguyễn Văn A</t>
   </si>
   <si>
-    <t>Chuyển kho</t>
-  </si>
-  <si>
-    <t>KT01</t>
-  </si>
-  <si>
-    <t>Nguyen Van C</t>
-  </si>
-  <si>
-    <t>Xe tải</t>
-  </si>
-  <si>
-    <t>WH01</t>
-  </si>
-  <si>
-    <t>WH02</t>
+    <t>VND</t>
+  </si>
+  <si>
+    <t>Trần Văn A</t>
+  </si>
+  <si>
+    <t>01002/HĐKG/2026</t>
+  </si>
+  <si>
+    <t>Xe</t>
+  </si>
+  <si>
+    <t>Tên đơn vị nhạp 1</t>
+  </si>
+  <si>
+    <t>Địa chỉ kho nhập 1</t>
   </si>
   <si>
     <t>sản phẩm 1</t>
@@ -168,28 +194,37 @@
     <t>CAI</t>
   </si>
   <si>
+    <t>200000</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
     <t>sản phẩm 2</t>
   </si>
   <si>
-    <t>Nguyễn Văn B</t>
-  </si>
-  <si>
-    <t>KT02</t>
-  </si>
-  <si>
-    <t>Nguyen Van D</t>
-  </si>
-  <si>
-    <t>xxx@gmail.com</t>
+    <t>100000</t>
+  </si>
+  <si>
+    <t>Trần Văn B</t>
+  </si>
+  <si>
+    <t>Tàu</t>
+  </si>
+  <si>
+    <t>Tên đơn vị nhạp 2</t>
+  </si>
+  <si>
+    <t>Địa chỉ kho nhập 2</t>
   </si>
   <si>
     <t>sp1</t>
   </si>
   <si>
     <t>gói</t>
+  </si>
+  <si>
+    <t>50000</t>
   </si>
   <si>
     <t>END</t>
@@ -287,8 +322,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -436,7 +472,7 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="36">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -451,7 +487,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
+        <fgColor theme="9" tint="0.8"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -626,12 +662,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -772,26 +802,26 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -905,42 +935,56 @@
     <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="1" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -950,12 +994,12 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1290,263 +1334,283 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Y5"/>
+  <dimension ref="A1:AA5"/>
   <sheetFormatPr defaultColWidth="25.4571428571429" defaultRowHeight="16.5" outlineLevelRow="4"/>
   <cols>
-    <col min="1" max="5" width="25.4571428571429" style="3"/>
-    <col min="6" max="6" width="26.4571428571429" style="3" customWidth="1"/>
-    <col min="7" max="7" width="25.4571428571429" style="3"/>
-    <col min="8" max="8" width="30.8190476190476" style="3" customWidth="1"/>
-    <col min="9" max="9" width="29.4571428571429" style="3" customWidth="1"/>
-    <col min="10" max="13" width="29.1809523809524" style="3" customWidth="1"/>
-    <col min="14" max="18" width="25.4571428571429" style="3"/>
-    <col min="19" max="23" width="25.4571428571429" style="4"/>
-    <col min="24" max="24" width="25.4571428571429" style="5"/>
-    <col min="25" max="25" width="25.4571428571429" style="4"/>
-    <col min="26" max="16384" width="25.4571428571429" style="6"/>
+    <col min="1" max="2" width="25.4571428571429" style="3"/>
+    <col min="3" max="3" width="25.4571428571429" style="4"/>
+    <col min="4" max="4" width="33.7142857142857" style="3" customWidth="1"/>
+    <col min="5" max="5" width="25.4571428571429" style="4"/>
+    <col min="6" max="6" width="29.8571428571429" style="3" customWidth="1"/>
+    <col min="7" max="7" width="28" style="3" customWidth="1"/>
+    <col min="8" max="8" width="30.8571428571429" style="4" customWidth="1"/>
+    <col min="9" max="9" width="32.4285714285714" style="3" customWidth="1"/>
+    <col min="10" max="10" width="27.1428571428571" style="3" customWidth="1"/>
+    <col min="11" max="22" width="25.4571428571429" style="3"/>
+    <col min="23" max="26" width="25.4571428571429" style="5"/>
+    <col min="27" max="27" width="25.4571428571429" style="6"/>
+    <col min="28" max="16384" width="25.4571428571429" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" s="2" customFormat="1" spans="1:25">
-      <c r="A1" s="7" t="s">
+    <row r="1" s="2" customFormat="1" spans="1:27">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="L1" s="10" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="N1" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="10" t="s">
+      <c r="O1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="10" t="s">
+      <c r="P1" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="Q1" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="R1" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="S1" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="12" t="s">
+      <c r="T1" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="10" t="s">
+      <c r="U1" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="10" t="s">
+      <c r="V1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="10" t="s">
+      <c r="W1" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="10" t="s">
+      <c r="X1" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" s="12" t="s">
+      <c r="Y1" s="13" t="s">
         <v>24</v>
       </c>
+      <c r="Z1" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="13" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="2" spans="1:24">
-      <c r="A2" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="3" t="s">
+    <row r="2" spans="1:27">
+      <c r="A2" s="17" t="s">
         <v>27</v>
       </c>
+      <c r="B2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="D2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="N2" s="3"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W2" s="5">
+        <v>1</v>
+      </c>
+      <c r="X2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y2" s="5">
+        <f t="shared" ref="Y2:Y4" si="0">W2*X2</f>
+        <v>200000</v>
+      </c>
+      <c r="Z2" s="5">
+        <v>1</v>
+      </c>
+      <c r="AA2" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27">
+      <c r="A3" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="U3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="V3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="W3" s="5">
+        <v>2</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="Y3" s="5">
+        <f t="shared" si="0"/>
+        <v>200000</v>
+      </c>
+      <c r="Z3" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:27">
+      <c r="A4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F2" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="G2" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J2" s="3" t="s">
+      <c r="F4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="G4" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="O2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q2" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="R2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="S2" s="4">
+      <c r="H4" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="N4" s="3"/>
+      <c r="O4" s="16"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="W4" s="5">
+        <v>12</v>
+      </c>
+      <c r="X4" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y4" s="5">
+        <f t="shared" si="0"/>
+        <v>600000</v>
+      </c>
+      <c r="Z4" s="5">
         <v>1</v>
       </c>
-      <c r="U2" s="4">
-        <v>0</v>
-      </c>
-      <c r="V2" s="4">
-        <f t="shared" ref="V2:V3" si="0">S2*U2</f>
-        <v>0</v>
-      </c>
-      <c r="W2" s="4">
-        <v>0</v>
-      </c>
-      <c r="X2" s="5">
-        <v>1</v>
+      <c r="AA4" s="6" t="s">
+        <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
-      <c r="A3" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="R3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="S3" s="4">
-        <v>2</v>
-      </c>
-      <c r="U3" s="4">
-        <v>0</v>
-      </c>
-      <c r="V3" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="W3" s="4">
-        <v>0</v>
-      </c>
-      <c r="X3" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24">
-      <c r="A4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="N4" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="Q4" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="R4" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="S4" s="4">
-        <v>12</v>
-      </c>
-      <c r="U4" s="4">
-        <v>0</v>
-      </c>
-      <c r="V4" s="4">
-        <v>0</v>
-      </c>
-      <c r="W4" s="4">
-        <v>0</v>
-      </c>
-      <c r="X4" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:27">
       <c r="A5" s="3" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="N4" r:id="rId3" display="xxx@gmail.com"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait"/>
   <headerFooter/>
@@ -1565,47 +1629,47 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="B2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="B3" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update some label and template for pxk
</commit_message>
<xml_diff>
--- a/hddt-SES/src/main/resources/static/agent/MauUpload_PXK_HKGDL_TT78.xlsx
+++ b/hddt-SES/src/main/resources/static/agent/MauUpload_PXK_HKGDL_TT78.xlsx
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="60">
   <si>
     <t>Mã phiếu(*)</t>
   </si>
@@ -83,7 +83,7 @@
     <t>Ngày lập (*)</t>
   </si>
   <si>
-    <t>Họ và tên người xuất kho (*)</t>
+    <t>Họ và tên người xuất kho</t>
   </si>
   <si>
     <t>Loại tiền (*)</t>
@@ -164,9 +164,6 @@
     <t>12/05/2026</t>
   </si>
   <si>
-    <t>Nguyễn Văn A</t>
-  </si>
-  <si>
     <t>VND</t>
   </si>
   <si>
@@ -179,9 +176,6 @@
     <t>Xe</t>
   </si>
   <si>
-    <t>Tên đơn vị nhạp 1</t>
-  </si>
-  <si>
     <t>Địa chỉ kho nhập 1</t>
   </si>
   <si>
@@ -210,9 +204,6 @@
   </si>
   <si>
     <t>Tàu</t>
-  </si>
-  <si>
-    <t>Tên đơn vị nhạp 2</t>
   </si>
   <si>
     <t>Địa chỉ kho nhập 2</t>
@@ -1362,7 +1353,7 @@
       <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="9" t="s">
@@ -1445,54 +1436,42 @@
       <c r="C2" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>33</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>29</v>
       </c>
       <c r="I2" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M2" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="N2" s="3"/>
       <c r="O2" s="15"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
       <c r="S2" s="3" t="s">
         <v>27</v>
       </c>
       <c r="T2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="U2" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="V2" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="U2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="V2" s="3" t="s">
-        <v>39</v>
       </c>
       <c r="W2" s="5">
         <v>1</v>
       </c>
       <c r="X2" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="Y2" s="5">
         <f t="shared" ref="Y2:Y4" si="0">W2*X2</f>
@@ -1510,22 +1489,22 @@
         <v>27</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="U3" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="W3" s="5">
         <v>2</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Y3" s="5">
         <f t="shared" si="0"/>
@@ -1537,7 +1516,7 @@
     </row>
     <row r="4" spans="1:27">
       <c r="A4" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>28</v>
@@ -1545,54 +1524,42 @@
       <c r="C4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>31</v>
-      </c>
       <c r="F4" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>29</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="N4" s="3"/>
+        <v>44</v>
+      </c>
       <c r="O4" s="16"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
       <c r="S4" s="3" t="s">
         <v>27</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="U4" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="V4" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="W4" s="5">
         <v>12</v>
       </c>
       <c r="X4" s="5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="Y4" s="5">
         <f t="shared" si="0"/>
@@ -1607,7 +1574,7 @@
     </row>
     <row r="5" spans="1:27">
       <c r="A5" s="3" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1629,47 +1596,47 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B4" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B5" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>